<commit_message>
fix(release): close v1.12.0 community evidence
</commit_message>
<xml_diff>
--- a/outputs/20260825-community-research/Hobbeast_kozossegi_allitasok_elfogadott_v1.12.0.xlsx
+++ b/outputs/20260825-community-research/Hobbeast_kozossegi_allitasok_elfogadott_v1.12.0.xlsx
@@ -2,10 +2,10 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Jegyzőkönyv" sheetId="1" r:id="R7649ad9a1e43401b"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Importálható" sheetId="2" r:id="R34870313bfe64733"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Forrásjegyzék" sheetId="3" r:id="R395e41200b9c42d6"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Lokalizációs séma" sheetId="4" r:id="R0db04f467ae24131"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Jegyzőkönyv" sheetId="1" r:id="R4fe5b158bdde40ee"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Importálható" sheetId="2" r:id="R3208a3e2e65c4f21"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Forrásjegyzék" sheetId="3" r:id="R992ffdb9cc22428e"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Lokalizációs séma" sheetId="4" r:id="R63cd690c77df4ee2"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -1972,7 +1972,7 @@
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R7ed54a7684664065"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rbb78040e96fc4322"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -2348,7 +2348,7 @@
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rdf99faa86c4b4e36"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R547a764419b84379"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -2365,7 +2365,7 @@
   <x:sheetData>
     <x:row r="1" ht="30" customHeight="1">
       <x:c r="A1" s="3" t="str">
-        <x:v>Lokalizációs adatmodell</x:v>
+        <x:v>Lokalizációs és publikációs adatmodell</x:v>
       </x:c>
       <x:c r="B1" s="3"/>
       <x:c r="C1" s="3"/>
@@ -2373,7 +2373,7 @@
     </x:row>
     <x:row r="2" ht="38" customHeight="1">
       <x:c r="A2" s="7" t="str">
-        <x:v>A stabil forrásrekord és a fordítható megjelenítési tartalom külön él; minden locale önálló review- és publikációs állapotot kaphat.</x:v>
+        <x:v>A stabil forrásrekord és a fordítható megjelenítési tartalom külön él. Nyilvánosan csak hash-egyező, locale-szinten is jóváhagyott és publikált fordítás jelenhet meg.</x:v>
       </x:c>
       <x:c r="B2" s="7"/>
       <x:c r="C2" s="7"/>
@@ -2393,74 +2393,130 @@
         <x:v>Szerep</x:v>
       </x:c>
     </x:row>
-    <x:row r="5" ht="58" customHeight="1">
+    <x:row r="5" ht="74" customHeight="1">
       <x:c r="A5" s="21" t="str">
         <x:v>community_research_claims</x:v>
       </x:c>
       <x:c r="B5" s="21" t="str">
-        <x:v>id, source_sequence_id, publication_year, source_url, doi, evidence_type, review_status, publication_status, is_active</x:v>
+        <x:v>id, canonical_key, source_sequence_id, original_locale, publication_year, source_url, doi, original_statement_sha256, review_status, publication_status, is_active, eligible_placements, editorial_metadata, reviewed_by, reviewed_at</x:v>
       </x:c>
       <x:c r="C5" s="21" t="str">
         <x:v>Nem</x:v>
       </x:c>
       <x:c r="D5" s="21" t="str">
-        <x:v>Stabil forrás-, audit- és lifecycle-adatok</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="6" ht="58" customHeight="1">
+        <x:v>Stabil forrás-, audit-, elhelyezési és claim-szintű lifecycle-adatok</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="6" ht="74" customHeight="1">
       <x:c r="A6" s="22" t="str">
         <x:v>community_research_claim_translations</x:v>
       </x:c>
       <x:c r="B6" s="22" t="str">
-        <x:v>claim_id, locale, statement_text, source_title, authors_display, translator_note</x:v>
+        <x:v>claim_id, locale, statement_text, source_title, source_container, authors_display, statement_sha256, review_status, publication_status, translator_note, reviewed_by, reviewed_at, is_original</x:v>
       </x:c>
       <x:c r="C6" s="22" t="str">
         <x:v>Igen</x:v>
       </x:c>
       <x:c r="D6" s="22" t="str">
-        <x:v>Locale-specifikus, változatlanul auditálható állítás és bibliográfiai megjelenítés</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="7" ht="58" customHeight="1">
+        <x:v>Locale-specifikus tartalom saját review/publikációs kapuval; szerkesztéskor automatikusan draft + pending_review</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="7" ht="74" customHeight="1">
       <x:c r="A7" s="22" t="str">
-        <x:v>community_research_claim_topics</x:v>
+        <x:v>community_research_topics</x:v>
       </x:c>
       <x:c r="B7" s="22" t="str">
-        <x:v>claim_id, topic_key</x:v>
+        <x:v>topic_key</x:v>
       </x:c>
       <x:c r="C7" s="22" t="str">
         <x:v>Nem</x:v>
       </x:c>
       <x:c r="D7" s="22" t="str">
+        <x:v>Stabil, nyelvfüggetlen keresési és kategorizálási kulcs</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="8" ht="74" customHeight="1">
+      <x:c r="A8" s="22" t="str">
+        <x:v>community_research_topic_translations</x:v>
+      </x:c>
+      <x:c r="B8" s="22" t="str">
+        <x:v>topic_key, locale, label</x:v>
+      </x:c>
+      <x:c r="C8" s="22" t="str">
+        <x:v>Igen</x:v>
+      </x:c>
+      <x:c r="D8" s="22" t="str">
+        <x:v>A tematikus címkék lokalizált megjelenítési neve</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="9" ht="74" customHeight="1">
+      <x:c r="A9" s="22" t="str">
+        <x:v>community_research_claim_topics</x:v>
+      </x:c>
+      <x:c r="B9" s="22" t="str">
+        <x:v>claim_id, topic_key</x:v>
+      </x:c>
+      <x:c r="C9" s="22" t="str">
+        <x:v>Nem</x:v>
+      </x:c>
+      <x:c r="D9" s="22" t="str">
         <x:v>Nyelvfüggetlen tematikus címkék</x:v>
       </x:c>
     </x:row>
-    <x:row r="8" ht="58" customHeight="1">
-      <x:c r="A8" s="22" t="str">
+    <x:row r="10" ht="74" customHeight="1">
+      <x:c r="A10" s="22" t="str">
         <x:v>community_research_claim_saves</x:v>
       </x:c>
-      <x:c r="B8" s="22" t="str">
+      <x:c r="B10" s="22" t="str">
         <x:v>user_id, claim_id, created_at</x:v>
       </x:c>
-      <x:c r="C8" s="22" t="str">
+      <x:c r="C10" s="22" t="str">
         <x:v>Nem</x:v>
       </x:c>
-      <x:c r="D8" s="22" t="str">
+      <x:c r="D10" s="22" t="str">
         <x:v>Felhasználónkénti szív + mentés; egyedi user/claim kulcs</x:v>
       </x:c>
     </x:row>
-    <x:row r="9" ht="58" customHeight="1">
-      <x:c r="A9" s="22" t="str">
+    <x:row r="11" ht="74" customHeight="1">
+      <x:c r="A11" s="22" t="str">
         <x:v>RPC</x:v>
       </x:c>
-      <x:c r="B9" s="22" t="str">
-        <x:v>get_random_community_research_claim(locale, placement, exclude_ids)</x:v>
-      </x:c>
-      <x:c r="C9" s="22" t="str">
+      <x:c r="B11" s="22" t="str">
+        <x:v>get_random_community_research_claim(locale, placement, random_cursor)</x:v>
+      </x:c>
+      <x:c r="C11" s="22" t="str">
         <x:v>—</x:v>
       </x:c>
-      <x:c r="D9" s="22" t="str">
-        <x:v>Csak approved + published + aktív rekord, locale-fallback és korlátozott random választás</x:v>
+      <x:c r="D11" s="22" t="str">
+        <x:v>Csak hash-hiteles, claim- és locale-szinten approved + published + aktív rekord; 1/N esélyű választás és biztonságos locale-fallback</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="12" ht="74" customHeight="1">
+      <x:c r="A12" s="22" t="str">
+        <x:v>RPC</x:v>
+      </x:c>
+      <x:c r="B12" s="22" t="str">
+        <x:v>set_community_research_claim_saved(claim_id, saved)</x:v>
+      </x:c>
+      <x:c r="C12" s="22" t="str">
+        <x:v>—</x:v>
+      </x:c>
+      <x:c r="D12" s="22" t="str">
+        <x:v>Bejelentkezett felhasználó szív + mentés művelete; a visszavonás akkor is engedett, ha a claim később lekerül</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="13" ht="74" customHeight="1">
+      <x:c r="A13" s="22" t="str">
+        <x:v>RPC</x:v>
+      </x:c>
+      <x:c r="B13" s="22" t="str">
+        <x:v>list_saved_community_research_claims(locale, limit, offset)</x:v>
+      </x:c>
+      <x:c r="C13" s="22" t="str">
+        <x:v>—</x:v>
+      </x:c>
+      <x:c r="D13" s="22" t="str">
+        <x:v>Privát, auth.uid()-hoz kötött, lapozott mentett könyvtár; maximum 25 rekord/kérés és csak publikálható tartalom</x:v>
       </x:c>
     </x:row>
   </x:sheetData>

</xml_diff>